<commit_message>
chore: update snapshots 2026-09-06
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1591"/>
+  <dimension ref="A1:H1601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -61866,6 +61866,386 @@
         </is>
       </c>
       <c r="H1591" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592" ht="15" customHeight="1">
+      <c r="A1592" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1592" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1592" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1592" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1592" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1592" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593" ht="15" customHeight="1">
+      <c r="A1593" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1593" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1593" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1593" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1593" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1593" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594" ht="15" customHeight="1">
+      <c r="A1594" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1594" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1594" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1594" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1594" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1594" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595" ht="15" customHeight="1">
+      <c r="A1595" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1595" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1595" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1595" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1595" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1595" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596" ht="15" customHeight="1">
+      <c r="A1596" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1596" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1596" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1596" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1596" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1596" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597" ht="15" customHeight="1">
+      <c r="A1597" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1597" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1597" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1597" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598" ht="15" customHeight="1">
+      <c r="A1598" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1598" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1598" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1598" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1598" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1598" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599" ht="15" customHeight="1">
+      <c r="A1599" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1599" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1599" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1599" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1599" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1599" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600" ht="15" customHeight="1">
+      <c r="A1600" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1600" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1600" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1600" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1600" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1600" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601" ht="15" customHeight="1">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>2026-09-06 12:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1601" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1601" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1601" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1601" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1601" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -62190,6 +62570,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1ee1bc38031cb4c46e45.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bbfacf51addf23f9c638.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.7d62cbffa5682629d6f7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e711d41c5d7899b1ee8c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bf58ba186e43f25b9111.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -62240,7 +62690,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -62265,7 +62715,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -62290,7 +62740,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -62315,7 +62765,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -62340,7 +62790,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -62365,7 +62815,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -62390,7 +62840,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -62415,7 +62865,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -62440,7 +62890,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -62465,7 +62915,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27 UTC</t>
+          <t>2026-09-06 12:40 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -62474,76 +62924,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1ee1bc38031cb4c46e45.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bbfacf51addf23f9c638.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.7d62cbffa5682629d6f7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e711d41c5d7899b1ee8c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bf58ba186e43f25b9111.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-07
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1601"/>
+  <dimension ref="A1:H1611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -62246,6 +62246,386 @@
         </is>
       </c>
       <c r="H1601" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602" ht="15" customHeight="1">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1602" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1602" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1602" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1602" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1602" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603" ht="15" customHeight="1">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1603" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1603" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1603" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1603" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1603" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604" ht="15" customHeight="1">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1604" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1604" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1604" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1604" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1604" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605" ht="15" customHeight="1">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1605" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1605" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1605" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1605" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1605" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606" ht="15" customHeight="1">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1606" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1606" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1606" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1606" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1606" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607" ht="15" customHeight="1">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1607" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1607" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1607" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1607" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1607" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608" ht="15" customHeight="1">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1608" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1608" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1608" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1608" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1608" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609" ht="15" customHeight="1">
+      <c r="A1609" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1609" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1609" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1609" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1609" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1609" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1609" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8e343e9401d5e7900424.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1609" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1ee1bc38031cb4c46e45.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bbfacf51addf23f9c638.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610" ht="15" customHeight="1">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1610" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1610" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1610" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1610" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1610" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611" ht="15" customHeight="1">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1611" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1611" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1611" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1611" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1611" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -62570,76 +62950,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1ee1bc38031cb4c46e45.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bbfacf51addf23f9c638.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.7d62cbffa5682629d6f7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e711d41c5d7899b1ee8c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bf58ba186e43f25b9111.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -62690,7 +63000,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -62715,7 +63025,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -62740,7 +63050,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -62765,7 +63075,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -62790,7 +63100,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -62815,7 +63125,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -62840,7 +63150,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -62865,7 +63175,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -62890,7 +63200,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -62915,7 +63225,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-06 12:40 UTC</t>
+          <t>2026-09-07 14:51 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -62924,6 +63234,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8e343e9401d5e7900424.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1ee1bc38031cb4c46e45.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bbfacf51addf23f9c638.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-08
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1611"/>
+  <dimension ref="A1:H1621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -62626,6 +62626,386 @@
         </is>
       </c>
       <c r="H1611" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612" ht="15" customHeight="1">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1612" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1612" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1612" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1612" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1612" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613" ht="15" customHeight="1">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1613" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1613" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1613" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614" ht="15" customHeight="1">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1614" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1614" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1614" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615" ht="15" customHeight="1">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1615" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1615" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1615" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616" ht="15" customHeight="1">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1616" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1616" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1616" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617" ht="15" customHeight="1">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1617" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1617" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1617" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618" ht="15" customHeight="1">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1618" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1618" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1618" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619" ht="15" customHeight="1">
+      <c r="A1619" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1619" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1619" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1619" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1619" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1619" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1619" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9689.716c18d2c386db397ab7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.2d3c6b7ea5b01630ed93.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.3efe8768184eed7c16a8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b8d626297ca64f5e02a8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9689.4344617c601ad099eb39.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1619" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8e343e9401d5e7900424.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620" ht="15" customHeight="1">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1620" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1620" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1620" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1620" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1620" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621" ht="15" customHeight="1">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1621" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1621" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1621" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1621" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -63000,7 +63380,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -63025,7 +63405,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -63050,7 +63430,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -63075,7 +63455,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -63100,7 +63480,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -63125,7 +63505,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -63150,7 +63530,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -63175,7 +63555,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -63200,7 +63580,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -63225,7 +63605,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-07 14:51 UTC</t>
+          <t>2026-09-08 13:21 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -63286,7 +63666,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8e343e9401d5e7900424.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9689.716c18d2c386db397ab7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.2d3c6b7ea5b01630ed93.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.3efe8768184eed7c16a8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b8d626297ca64f5e02a8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9689.4344617c601ad099eb39.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -63303,7 +63683,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1ee1bc38031cb4c46e45.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.bbfacf51addf23f9c638.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.c66a03a89c777ed97f63.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/79980.ea2eb91b5ea7f69df716.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/66507.4b11e24f89c8ef9baf5e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.f47c4dcacd8955c611f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/95154.234a2a8362226ec1f2f1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18982.050e663232a82d5a8372.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8e343e9401d5e7900424.js"&gt;&lt;/script&gt;&lt;link href="/style/css/79980.f8f9203cda8223740788.css" rel="stylesheet"&gt;&lt;link href="/style/css/18982.839cef121b1d8fbd564c.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.9e50c728a19482ae4272.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-24
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1771"/>
+  <dimension ref="A1:H1781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -68945,82 +68945,392 @@
         </is>
       </c>
     </row>
+    <row r="1772" ht="15" customHeight="1">
+      <c r="A1772" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1772" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1772" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1772" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1772" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1772" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1772" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773" ht="15" customHeight="1">
+      <c r="A1773" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1773" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1773" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1773" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1773" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1773" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1773" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774" ht="15" customHeight="1">
+      <c r="A1774" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1774" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1774" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1774" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1774" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1774" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1774" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775" ht="15" customHeight="1">
+      <c r="A1775" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1775" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1775" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1775" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1775" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1775" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1775" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776" ht="15" customHeight="1">
+      <c r="A1776" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1776" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1776" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1776" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1776" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1776" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1776" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777" ht="15" customHeight="1">
+      <c r="A1777" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1777" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1777" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1777" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1777" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1777" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1777" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778" ht="15" customHeight="1">
+      <c r="A1778" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1778" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1778" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1778" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1778" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1778" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1778" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779" ht="15" customHeight="1">
+      <c r="A1779" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1779" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1779" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1779" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1779" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1779" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1779" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.570c63468d1b20ff829b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.c8887e82d4e4e0c952d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b4410e07d650ed3d29ff.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1779" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45070.df21e60a0fafc90959ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.5aa6112ebce90055c72c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.dd3aa19dc9ccaf6411e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.de2e5117c09861b8ce77.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/49686.c390cdc5beebfe2c9080.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.545e04852d4a190e7fb3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/45070.634001c3db6038117801.css" rel="stylesheet"&gt;&lt;link href="/style/css/49686.d8c6ca69a07f12c9535d.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780" ht="15" customHeight="1">
+      <c r="A1780" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1780" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1780" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1780" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1780" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1780" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781" ht="15" customHeight="1">
+      <c r="A1781" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1781" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1781" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1781" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1781" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1781" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45070.df21e60a0fafc90959ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.5aa6112ebce90055c72c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.dd3aa19dc9ccaf6411e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.de2e5117c09861b8ce77.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/49686.c390cdc5beebfe2c9080.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.545e04852d4a190e7fb3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/45070.634001c3db6038117801.css" rel="stylesheet"&gt;&lt;link href="/style/css/49686.d8c6ca69a07f12c9535d.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45070.a26685583c0b2c652c72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.897d9d3dc7eac3be2914.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.dd3aa19dc9ccaf6411e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.de2e5117c09861b8ce77.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/49686.67bf72f1219d4ecf09ec.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.01c8651008d0ce16b75a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/45070.634001c3db6038117801.css" rel="stylesheet"&gt;&lt;link href="/style/css/49686.d8c6ca69a07f12c9535d.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.d9daca81ba7f337f6519.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -69192,179 +69502,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Sonobi</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2014616652, RESELLER, 98c21ef9a666c68b</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>anyclip.com, 001Te00000hfb7hIAA, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 5759, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, 5759, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>triplelift.com, 424, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>mediafuse.com, 403, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>benefit.media, 2268428, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#anyclip</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>nativo.com, 6077, RESELLER, 59521ca7cc5e9fee</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -69420,7 +69558,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -69445,7 +69583,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -69470,7 +69608,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -69495,7 +69633,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -69520,7 +69658,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -69545,7 +69683,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -69570,7 +69708,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -69595,7 +69733,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -69620,7 +69758,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -69645,7 +69783,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-23 14:06 UTC</t>
+          <t>2026-09-24 14:04 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -69654,6 +69792,248 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.570c63468d1b20ff829b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.c8887e82d4e4e0c952d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b4410e07d650ed3d29ff.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45070.df21e60a0fafc90959ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.5aa6112ebce90055c72c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.dd3aa19dc9ccaf6411e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.de2e5117c09861b8ce77.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/49686.c390cdc5beebfe2c9080.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.545e04852d4a190e7fb3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/45070.634001c3db6038117801.css" rel="stylesheet"&gt;&lt;link href="/style/css/49686.d8c6ca69a07f12c9535d.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Sonobi</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2014616652, RESELLER, 98c21ef9a666c68b</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>anyclip.com, 001Te00000hfb7hIAA, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 5759, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5759, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 424, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>mediafuse.com, 403, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>benefit.media, 2268428, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#anyclip</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>nativo.com, 6077, RESELLER, 59521ca7cc5e9fee</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-25
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1781"/>
+  <dimension ref="A1:H1791"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -69320,6 +69320,386 @@
         </is>
       </c>
       <c r="H1781" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782" ht="15" customHeight="1">
+      <c r="A1782" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1782" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1782" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1782" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1782" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1782" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783" ht="15" customHeight="1">
+      <c r="A1783" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1783" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1783" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1783" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1783" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1783" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784" ht="15" customHeight="1">
+      <c r="A1784" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1784" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1784" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1784" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1784" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1784" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785" ht="15" customHeight="1">
+      <c r="A1785" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1785" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1785" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1785" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1785" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1785" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786" ht="15" customHeight="1">
+      <c r="A1786" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1786" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1786" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1786" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1786" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1786" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787" ht="15" customHeight="1">
+      <c r="A1787" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1787" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1787" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1787" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1787" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1787" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788" ht="15" customHeight="1">
+      <c r="A1788" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1788" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1788" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1788" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1788" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1788" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789" ht="15" customHeight="1">
+      <c r="A1789" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1789" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1789" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1789" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1789" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1789" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1789" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1789" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.570c63468d1b20ff829b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.c8887e82d4e4e0c952d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b4410e07d650ed3d29ff.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790" ht="15" customHeight="1">
+      <c r="A1790" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1790" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1790" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1790" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1790" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1790" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791" ht="15" customHeight="1">
+      <c r="A1791" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1791" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1791" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1791" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1791" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1791" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -69558,7 +69938,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -69583,7 +69963,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -69608,7 +69988,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -69633,7 +70013,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -69658,7 +70038,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -69683,7 +70063,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -69708,7 +70088,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -69733,7 +70113,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -69758,7 +70138,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -69783,7 +70163,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-24 14:04 UTC</t>
+          <t>2026-09-25 14:27 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -69844,7 +70224,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.570c63468d1b20ff829b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.c8887e82d4e4e0c952d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b4410e07d650ed3d29ff.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -69861,7 +70241,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45070.df21e60a0fafc90959ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.5aa6112ebce90055c72c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.dd3aa19dc9ccaf6411e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.de2e5117c09861b8ce77.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/49686.c390cdc5beebfe2c9080.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.545e04852d4a190e7fb3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/45070.634001c3db6038117801.css" rel="stylesheet"&gt;&lt;link href="/style/css/49686.d8c6ca69a07f12c9535d.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.570c63468d1b20ff829b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.c8887e82d4e4e0c952d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b4410e07d650ed3d29ff.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-26
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1791"/>
+  <dimension ref="A1:H1801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -69700,6 +69700,386 @@
         </is>
       </c>
       <c r="H1791" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792" ht="15" customHeight="1">
+      <c r="A1792" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1792" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1792" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1792" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1792" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1792" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1793" ht="15" customHeight="1">
+      <c r="A1793" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1793" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1793" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1793" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1793" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1793" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794" ht="15" customHeight="1">
+      <c r="A1794" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1794" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1794" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1794" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1794" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1794" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795" ht="15" customHeight="1">
+      <c r="A1795" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1795" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1795" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1795" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1795" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1795" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796" ht="15" customHeight="1">
+      <c r="A1796" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1796" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1796" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1796" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1796" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1796" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797" ht="15" customHeight="1">
+      <c r="A1797" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1797" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1797" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1797" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1797" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1797" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1798" ht="15" customHeight="1">
+      <c r="A1798" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1798" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1798" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1798" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1798" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1798" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799" ht="15" customHeight="1">
+      <c r="A1799" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1799" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1799" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1799" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1799" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1799" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1799" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1799" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800" ht="15" customHeight="1">
+      <c r="A1800" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1800" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1800" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1800" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1800" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1800" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801" ht="15" customHeight="1">
+      <c r="A1801" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:38 UTC</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1801" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1801" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1801" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1801" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1801" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -69938,7 +70318,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -69963,7 +70343,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -69988,7 +70368,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -70013,7 +70393,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -70038,7 +70418,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -70063,7 +70443,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -70088,7 +70468,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -70113,7 +70493,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -70138,7 +70518,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -70163,7 +70543,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-25 14:27 UTC</t>
+          <t>2026-09-26 13:38 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -70224,7 +70604,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -70241,7 +70621,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.570c63468d1b20ff829b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.c8887e82d4e4e0c952d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b4410e07d650ed3d29ff.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-27
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1801"/>
+  <dimension ref="A1:H1811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -70080,6 +70080,386 @@
         </is>
       </c>
       <c r="H1801" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1802" ht="15" customHeight="1">
+      <c r="A1802" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1802" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1802" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1802" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1802" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1802" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803" ht="15" customHeight="1">
+      <c r="A1803" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1803" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1803" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1803" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1803" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1803" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804" ht="15" customHeight="1">
+      <c r="A1804" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1804" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1804" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1804" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1804" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1804" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805" ht="15" customHeight="1">
+      <c r="A1805" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1805" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1805" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1805" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1805" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1805" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806" ht="15" customHeight="1">
+      <c r="A1806" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1806" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1806" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1806" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1806" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1806" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807" ht="15" customHeight="1">
+      <c r="A1807" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1807" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1807" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1807" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1807" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1807" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808" ht="15" customHeight="1">
+      <c r="A1808" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1808" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1808" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1808" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1808" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1808" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809" ht="15" customHeight="1">
+      <c r="A1809" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1809" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1809" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1809" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1809" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1809" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810" ht="15" customHeight="1">
+      <c r="A1810" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1810" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1810" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1810" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1810" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1810" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811" ht="15" customHeight="1">
+      <c r="A1811" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1811" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1811" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1811" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1811" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1811" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -70268,6 +70648,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -70318,7 +70768,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -70343,7 +70793,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -70368,7 +70818,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -70393,7 +70843,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -70418,7 +70868,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -70443,7 +70893,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -70468,7 +70918,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -70493,7 +70943,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -70518,7 +70968,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -70543,7 +70993,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-26 13:38 UTC</t>
+          <t>2026-09-27 14:35 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -70552,76 +71002,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-28
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1811"/>
+  <dimension ref="A1:H1821"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -70460,6 +70460,386 @@
         </is>
       </c>
       <c r="H1811" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812" ht="15" customHeight="1">
+      <c r="A1812" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1812" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1812" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1812" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1812" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1812" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813" ht="15" customHeight="1">
+      <c r="A1813" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1813" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1813" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1813" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1813" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1813" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1814" ht="15" customHeight="1">
+      <c r="A1814" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1814" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1814" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1814" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1814" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1814" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815" ht="15" customHeight="1">
+      <c r="A1815" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1815" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1815" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1815" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1815" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1815" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816" ht="15" customHeight="1">
+      <c r="A1816" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1816" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1816" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1816" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1816" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1816" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817" ht="15" customHeight="1">
+      <c r="A1817" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1817" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1817" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1817" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1817" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1817" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818" ht="15" customHeight="1">
+      <c r="A1818" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1818" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1818" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1818" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1818" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1818" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819" ht="15" customHeight="1">
+      <c r="A1819" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1819" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1819" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1819" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1819" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1819" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1819" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.06004e6adc3188ffab72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.3e9bfa576b343202b158.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e2dee9d8bcb5a3122c90.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1819" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820" ht="15" customHeight="1">
+      <c r="A1820" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1820" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1820" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1820" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1820" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1820" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821" ht="15" customHeight="1">
+      <c r="A1821" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1821" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1821" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1821" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1821" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1821" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -70648,76 +71028,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.a9ae7468df5a8130135a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.5bfc80e8dfd5580f6384.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.243c553047d6b2f2db03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -70768,7 +71078,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -70793,7 +71103,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -70818,7 +71128,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -70843,7 +71153,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -70868,7 +71178,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -70893,7 +71203,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -70918,7 +71228,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -70943,7 +71253,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -70968,7 +71278,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -70993,7 +71303,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-27 14:35 UTC</t>
+          <t>2026-09-28 17:25 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -71002,6 +71312,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.06004e6adc3188ffab72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.3e9bfa576b343202b158.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e2dee9d8bcb5a3122c90.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-29
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1821"/>
+  <dimension ref="A1:H1831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -70840,6 +70840,386 @@
         </is>
       </c>
       <c r="H1821" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822" ht="15" customHeight="1">
+      <c r="A1822" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1822" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1822" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1822" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1822" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1822" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823" ht="15" customHeight="1">
+      <c r="A1823" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1823" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1823" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1823" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1823" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1823" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1824" ht="15" customHeight="1">
+      <c r="A1824" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1824" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1824" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1824" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1824" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1824" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825" ht="15" customHeight="1">
+      <c r="A1825" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1825" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1825" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1825" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1825" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1825" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826" ht="15" customHeight="1">
+      <c r="A1826" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1826" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1826" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1826" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1826" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1826" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827" ht="15" customHeight="1">
+      <c r="A1827" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1827" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1827" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1827" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1827" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1827" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828" ht="15" customHeight="1">
+      <c r="A1828" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1828" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1828" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1828" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1828" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1828" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829" ht="15" customHeight="1">
+      <c r="A1829" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1829" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1829" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1829" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1829" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1829" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1829" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d24a01ed6b02c0ac447d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.91feb4561c17e8ccee96.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1829" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.06004e6adc3188ffab72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.3e9bfa576b343202b158.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e2dee9d8bcb5a3122c90.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830" ht="15" customHeight="1">
+      <c r="A1830" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1830" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1830" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1830" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1830" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1830" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831" ht="15" customHeight="1">
+      <c r="A1831" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:25 UTC</t>
+        </is>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1831" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1831" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1831" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1831" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1831" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -71078,7 +71458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -71103,7 +71483,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -71128,7 +71508,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -71153,7 +71533,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -71178,7 +71558,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -71203,7 +71583,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -71228,7 +71608,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -71253,7 +71633,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -71278,7 +71658,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -71303,7 +71683,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-28 17:25 UTC</t>
+          <t>2026-09-29 15:25 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -71364,7 +71744,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.06004e6adc3188ffab72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.3e9bfa576b343202b158.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e2dee9d8bcb5a3122c90.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d24a01ed6b02c0ac447d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.91feb4561c17e8ccee96.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -71381,7 +71761,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.01cc91179d7845ff430d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.0b800be1a9d8517c7c33.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.2aca647041a2d49ab5e3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.06004e6adc3188ffab72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.3e9bfa576b343202b158.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e2dee9d8bcb5a3122c90.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-09-30
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1831"/>
+  <dimension ref="A1:H1841"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -71220,6 +71220,386 @@
         </is>
       </c>
       <c r="H1831" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832" ht="15" customHeight="1">
+      <c r="A1832" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1832" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1832" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1832" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1832" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1832" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833" ht="15" customHeight="1">
+      <c r="A1833" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1833" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1833" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1833" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1833" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1833" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834" ht="15" customHeight="1">
+      <c r="A1834" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1834" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1834" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1834" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1834" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1834" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835" ht="15" customHeight="1">
+      <c r="A1835" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1835" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1835" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1835" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1835" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1835" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836" ht="15" customHeight="1">
+      <c r="A1836" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1836" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1836" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1836" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1836" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1836" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837" ht="15" customHeight="1">
+      <c r="A1837" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1837" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1837" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1837" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1837" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1837" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838" ht="15" customHeight="1">
+      <c r="A1838" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1838" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1838" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1838" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1838" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1838" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839" ht="15" customHeight="1">
+      <c r="A1839" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1839" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1839" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1839" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1839" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1839" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1839" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.264b133602defae6b8d0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1839" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d24a01ed6b02c0ac447d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.91feb4561c17e8ccee96.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840" ht="15" customHeight="1">
+      <c r="A1840" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1840" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1840" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1840" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1840" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1840" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841" ht="15" customHeight="1">
+      <c r="A1841" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1841" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1841" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1841" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1841" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1841" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -71458,7 +71838,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -71483,7 +71863,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -71508,7 +71888,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -71533,7 +71913,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -71558,7 +71938,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -71583,7 +71963,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -71608,7 +71988,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -71633,7 +72013,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -71658,7 +72038,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -71683,7 +72063,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-29 15:25 UTC</t>
+          <t>2026-09-30 15:42 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -71744,7 +72124,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d24a01ed6b02c0ac447d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.91feb4561c17e8ccee96.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.264b133602defae6b8d0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -71761,7 +72141,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.419c9f1bfc6ef0d8dd92.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.3cbea42edb89a5b6337b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.a0128552046213f23329.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/93627.74e4ef94ac859437144e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.a98bc8cb1642d637d37e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.adbe951eaf990858267a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.06004e6adc3188ffab72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/64296.3e9bfa576b343202b158.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e2dee9d8bcb5a3122c90.js"&gt;&lt;/script&gt;&lt;link href="/style/css/93627.181ece40b08385311a7c.css" rel="stylesheet"&gt;&lt;link href="/style/css/64296.445266e3756b2736808f.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f00770abbd8d9d7ac9e8.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d24a01ed6b02c0ac447d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.91feb4561c17e8ccee96.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-01
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1841"/>
+  <dimension ref="A1:H1851"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -71600,6 +71600,386 @@
         </is>
       </c>
       <c r="H1841" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842" ht="15" customHeight="1">
+      <c r="A1842" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1842" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1842" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1842" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1842" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1842" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843" ht="15" customHeight="1">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1843" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1843" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1843" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1843" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1843" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844" ht="15" customHeight="1">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1844" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1844" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1844" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1844" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1844" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845" ht="15" customHeight="1">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1845" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1845" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1845" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1845" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1845" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846" ht="15" customHeight="1">
+      <c r="A1846" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1846" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1846" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1846" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1846" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1846" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847" ht="15" customHeight="1">
+      <c r="A1847" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1847" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1847" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1847" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1847" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1847" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848" ht="15" customHeight="1">
+      <c r="A1848" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1848" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1848" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1848" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1848" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1848" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849" ht="15" customHeight="1">
+      <c r="A1849" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1849" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1849" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1849" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1849" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1849" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1849" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1849" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.264b133602defae6b8d0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850" ht="15" customHeight="1">
+      <c r="A1850" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1850" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1850" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1850" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1850" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1850" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851" ht="15" customHeight="1">
+      <c r="A1851" t="inlineStr">
+        <is>
+          <t>2026-10-01 16:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1851" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1851" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1851" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1851" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1851" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -71838,7 +72218,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -71863,7 +72243,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -71888,7 +72268,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -71913,7 +72293,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -71938,7 +72318,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -71963,7 +72343,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -71988,7 +72368,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -72013,7 +72393,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -72038,7 +72418,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -72063,7 +72443,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-30 15:42 UTC</t>
+          <t>2026-10-01 16:03 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -72124,7 +72504,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.264b133602defae6b8d0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -72141,7 +72521,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d24a01ed6b02c0ac447d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.91feb4561c17e8ccee96.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.264b133602defae6b8d0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-02
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1851"/>
+  <dimension ref="A1:H1861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -71980,6 +71980,386 @@
         </is>
       </c>
       <c r="H1851" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852" ht="15" customHeight="1">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1852" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1852" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1852" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1852" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1852" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853" ht="15" customHeight="1">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1853" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1853" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1853" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1853" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1853" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854" ht="15" customHeight="1">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1854" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1854" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1854" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1854" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1854" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855" ht="15" customHeight="1">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1855" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1855" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1855" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1855" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1855" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856" ht="15" customHeight="1">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1856" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1856" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1856" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1856" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1856" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857" ht="15" customHeight="1">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1857" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1857" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1857" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1857" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1857" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858" ht="15" customHeight="1">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1858" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1858" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1858" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1858" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1858" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859" ht="15" customHeight="1">
+      <c r="A1859" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1859" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1859" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1859" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1859" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1859" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1859" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1859" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860" ht="15" customHeight="1">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1860" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1860" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1860" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1860" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1860" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861" ht="15" customHeight="1">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27 UTC</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1861" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1861" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1861" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1861" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1861" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -72218,7 +72598,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -72243,7 +72623,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -72268,7 +72648,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -72293,7 +72673,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -72318,7 +72698,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -72343,7 +72723,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -72368,7 +72748,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -72393,7 +72773,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -72418,7 +72798,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -72443,7 +72823,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-01 16:03 UTC</t>
+          <t>2026-10-02 15:27 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -72504,7 +72884,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -72521,7 +72901,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.915ecab62e4e8725ef75.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.4bebf3fe17e71cd58ff8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.24e1209c02e864b450bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/38837.9259dc672ad697f60ed7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/23617.99b5a965110df244ba10.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.9b053d441a81eb78b63e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a223af4c06f70aeed231.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/31533.3f911f5c480b4a35e33e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.264b133602defae6b8d0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/38837.e54fc2aa5ace4bff3e9f.css" rel="stylesheet"&gt;&lt;link href="/style/css/31533.fba9e980f5e3534dcdd6.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-03
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1861"/>
+  <dimension ref="A1:H1871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -72360,6 +72360,386 @@
         </is>
       </c>
       <c r="H1861" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862" ht="15" customHeight="1">
+      <c r="A1862" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1862" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1862" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1862" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1862" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1862" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863" ht="15" customHeight="1">
+      <c r="A1863" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1863" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1863" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1863" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1863" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1863" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864" ht="15" customHeight="1">
+      <c r="A1864" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1864" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1864" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1864" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1864" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1864" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865" ht="15" customHeight="1">
+      <c r="A1865" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1865" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1865" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1865" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1865" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1865" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866" ht="15" customHeight="1">
+      <c r="A1866" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1866" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1866" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1866" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1866" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1866" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867" ht="15" customHeight="1">
+      <c r="A1867" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1867" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1867" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1867" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1867" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1867" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868" ht="15" customHeight="1">
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1868" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1868" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1868" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1868" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1868" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869" ht="15" customHeight="1">
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1869" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1869" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1869" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1869" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1869" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870" ht="15" customHeight="1">
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1870" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1870" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1870" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1870" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1870" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871" ht="15" customHeight="1">
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1871" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1871" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1871" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1871" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1871" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -72548,6 +72928,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -72598,7 +73048,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -72623,7 +73073,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -72648,7 +73098,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -72673,7 +73123,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -72698,7 +73148,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -72723,7 +73173,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -72748,7 +73198,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -72773,7 +73223,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -72798,7 +73248,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -72823,7 +73273,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-02 15:27 UTC</t>
+          <t>2026-10-03 14:10 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -72832,76 +73282,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-04
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1871"/>
+  <dimension ref="A1:H1881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -72740,6 +72740,386 @@
         </is>
       </c>
       <c r="H1871" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872" ht="15" customHeight="1">
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1872" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1872" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1872" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1872" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1872" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873" ht="15" customHeight="1">
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1873" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1873" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1873" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1873" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1873" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874" ht="15" customHeight="1">
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1874" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1874" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1874" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1874" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1874" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1875" ht="15" customHeight="1">
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1875" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1875" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1875" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1875" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1875" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876" ht="15" customHeight="1">
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1876" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1876" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1876" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1876" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1876" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877" ht="15" customHeight="1">
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1877" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1877" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1877" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1877" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1877" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878" ht="15" customHeight="1">
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1878" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1878" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1878" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1878" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1878" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1879" ht="15" customHeight="1">
+      <c r="A1879" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1879" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1879" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1879" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1879" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1879" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1879" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1879" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1880" ht="15" customHeight="1">
+      <c r="A1880" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1880" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1880" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1880" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1880" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1880" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1880" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1880" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881" ht="15" customHeight="1">
+      <c r="A1881" t="inlineStr">
+        <is>
+          <t>2026-10-04 14:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1881" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1881" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1881" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1881" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1881" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1881" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1881" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -73048,7 +73428,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -73073,7 +73453,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -73098,7 +73478,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -73123,7 +73503,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -73148,7 +73528,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -73173,7 +73553,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -73198,7 +73578,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -73223,7 +73603,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -73248,7 +73628,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -73273,7 +73653,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-03 14:10 UTC</t>
+          <t>2026-10-04 14:39 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-05
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1881"/>
+  <dimension ref="A1:H1891"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -73120,6 +73120,386 @@
         </is>
       </c>
       <c r="H1881" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1882" ht="15" customHeight="1">
+      <c r="A1882" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1882" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1882" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1882" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1882" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1882" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1882" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1882" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1883" ht="15" customHeight="1">
+      <c r="A1883" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1883" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1883" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1883" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1883" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1883" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1883" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1883" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1884" ht="15" customHeight="1">
+      <c r="A1884" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1884" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1884" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1884" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1884" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1884" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1884" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1884" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1885" ht="15" customHeight="1">
+      <c r="A1885" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1885" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1885" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1885" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1885" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1885" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1885" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1885" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1886" ht="15" customHeight="1">
+      <c r="A1886" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1886" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1886" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1886" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1886" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1886" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1886" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1886" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1887" ht="15" customHeight="1">
+      <c r="A1887" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1887" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1887" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1887" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1887" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1887" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1887" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1887" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1888" ht="15" customHeight="1">
+      <c r="A1888" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1888" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1888" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1888" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1888" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1888" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1888" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1888" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1889" ht="15" customHeight="1">
+      <c r="A1889" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1889" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1889" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1889" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1889" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1889" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1889" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.7e287fc1177f6b14339a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.cb6aa9a249ad29dcd58a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.2528d70ea54aa0f87758.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.4ea618025394f60cffcb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1889" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1890" ht="15" customHeight="1">
+      <c r="A1890" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1890" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1890" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1890" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1890" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1890" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1890" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1890" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1891" ht="15" customHeight="1">
+      <c r="A1891" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1891" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1891" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1891" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1891" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1891" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1891" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1891" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -73308,76 +73688,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.ae5571c78802a1362c1e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.5b2210cc27b78d4a26bd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.219460f16696e460db46.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.c3971665f11558403b03.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77d5350384bdf88f5157.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.e20e3e8bef755394062c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -73428,7 +73738,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -73453,7 +73763,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -73478,7 +73788,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -73503,7 +73813,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -73528,7 +73838,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -73553,7 +73863,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -73578,7 +73888,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -73603,7 +73913,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -73628,7 +73938,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -73653,7 +73963,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-04 14:39 UTC</t>
+          <t>2026-10-05 18:01 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -73662,6 +73972,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.7e287fc1177f6b14339a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.cb6aa9a249ad29dcd58a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.2528d70ea54aa0f87758.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.4ea618025394f60cffcb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-06
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1891"/>
+  <dimension ref="A1:H1901"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -73500,6 +73500,386 @@
         </is>
       </c>
       <c r="H1891" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1892" ht="15" customHeight="1">
+      <c r="A1892" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1892" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1892" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1892" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1892" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1892" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1892" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1892" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1893" ht="15" customHeight="1">
+      <c r="A1893" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1893" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1893" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1893" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1893" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1893" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1893" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1893" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1894" ht="15" customHeight="1">
+      <c r="A1894" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1894" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1894" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1894" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1894" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1894" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1894" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1894" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1895" ht="15" customHeight="1">
+      <c r="A1895" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1895" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1895" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1895" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1895" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1895" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1895" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1895" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1896" ht="15" customHeight="1">
+      <c r="A1896" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1896" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1896" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1896" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1896" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1896" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1896" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1896" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1897" ht="15" customHeight="1">
+      <c r="A1897" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1897" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1897" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1897" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1897" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1897" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1897" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1897" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1898" ht="15" customHeight="1">
+      <c r="A1898" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1898" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1898" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1898" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1898" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1898" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1898" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1898" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1899" ht="15" customHeight="1">
+      <c r="A1899" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1899" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1899" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1899" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1899" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1899" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1899" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.1f45837ebf350fcb1b06.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.b04da66fc7640a4a5b88.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.aeeaa96fcd059dc802f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.3e22eab7d3ff25b86b7f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b958de8eb80c530d128.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.7e97b3c950c96ab7e1af.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1899" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.7e287fc1177f6b14339a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.cb6aa9a249ad29dcd58a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.2528d70ea54aa0f87758.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.4ea618025394f60cffcb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1900" ht="15" customHeight="1">
+      <c r="A1900" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1900" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1900" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1900" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1900" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1900" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1900" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1900" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1901" ht="15" customHeight="1">
+      <c r="A1901" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:43 UTC</t>
+        </is>
+      </c>
+      <c r="B1901" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1901" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1901" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1901" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1901" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1901" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1901" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -73738,7 +74118,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -73763,7 +74143,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -73788,7 +74168,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -73813,7 +74193,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -73838,7 +74218,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -73863,7 +74243,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -73888,7 +74268,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -73913,7 +74293,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -73938,7 +74318,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -73963,7 +74343,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-05 18:01 UTC</t>
+          <t>2026-10-06 15:43 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -74024,7 +74404,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.7e287fc1177f6b14339a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.cb6aa9a249ad29dcd58a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.2528d70ea54aa0f87758.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.4ea618025394f60cffcb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.1f45837ebf350fcb1b06.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.b04da66fc7640a4a5b88.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.aeeaa96fcd059dc802f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.3e22eab7d3ff25b86b7f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b958de8eb80c530d128.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.7e97b3c950c96ab7e1af.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -74041,7 +74421,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.64acaf602e838ab61f85.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.89f5906060f05e43a20e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.efd5da8f801d1683ff19.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c2e1ecd9d4add07c1df2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.7e287fc1177f6b14339a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.cb6aa9a249ad29dcd58a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.2528d70ea54aa0f87758.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.4ea618025394f60cffcb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-10-07
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1901"/>
+  <dimension ref="A1:H1911"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -73880,6 +73880,386 @@
         </is>
       </c>
       <c r="H1901" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1902" ht="15" customHeight="1">
+      <c r="A1902" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1902" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1902" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1902" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1902" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1902" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1902" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1902" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1903" ht="15" customHeight="1">
+      <c r="A1903" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1903" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1903" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1903" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1903" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1903" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1903" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1903" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1904" ht="15" customHeight="1">
+      <c r="A1904" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1904" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1904" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1904" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1904" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1904" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1904" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1904" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1905" ht="15" customHeight="1">
+      <c r="A1905" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1905" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1905" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1905" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1905" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1905" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1905" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1905" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1906" ht="15" customHeight="1">
+      <c r="A1906" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1906" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1906" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1906" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1906" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1906" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1906" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1906" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1907" ht="15" customHeight="1">
+      <c r="A1907" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1907" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1907" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1907" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1907" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1907" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1907" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1907" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1908" ht="15" customHeight="1">
+      <c r="A1908" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1908" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1908" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1908" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1908" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1908" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1908" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1908" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1909" ht="15" customHeight="1">
+      <c r="A1909" s="3" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1909" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1909" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1909" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1909" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1909" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1909" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.5acc0961104bc0f338ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.3c5a374478df5356ffbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.531b29ba2f97b6bc4fbd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/76171.df2c0eaec0d30eca9b61.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.a94970f05b4d5d8b9a8e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.912df29ab52e5699256f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/76171.7e71223a5b3c0d0c05a1.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.2bdd16b6ae60954db24f.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1909" s="3" t="inlineStr">
+        <is>
+          <t>(no section): }&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.1f45837ebf350fcb1b06.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.b04da66fc7640a4a5b88.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.aeeaa96fcd059dc802f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.3e22eab7d3ff25b86b7f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b958de8eb80c530d128.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.7e97b3c950c96ab7e1af.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1910" ht="15" customHeight="1">
+      <c r="A1910" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1910" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1910" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1910" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1910" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1910" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1910" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1910" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1911" ht="15" customHeight="1">
+      <c r="A1911" t="inlineStr">
+        <is>
+          <t>2026-10-07 16:08 UTC</t>
+        </is>
+      </c>
+      <c r="B1911" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1911" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1911" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1911" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1911" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1911" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1911" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -74118,7 +74498,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -74143,7 +74523,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -74168,7 +74548,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -74193,7 +74573,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -74218,7 +74598,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -74243,7 +74623,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -74268,7 +74648,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -74293,7 +74673,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -74318,7 +74698,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -74343,7 +74723,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-06 15:43 UTC</t>
+          <t>2026-10-07 16:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -74404,7 +74784,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.1f45837ebf350fcb1b06.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.b04da66fc7640a4a5b88.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.aeeaa96fcd059dc802f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.3e22eab7d3ff25b86b7f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b958de8eb80c530d128.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.7e97b3c950c96ab7e1af.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.5acc0961104bc0f338ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.3c5a374478df5356ffbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.531b29ba2f97b6bc4fbd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/76171.df2c0eaec0d30eca9b61.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.a94970f05b4d5d8b9a8e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.912df29ab52e5699256f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/76171.7e71223a5b3c0d0c05a1.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.2bdd16b6ae60954db24f.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -74421,7 +74801,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.346a1e7ea39ad05269b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.c4c49a5a54f0010cb237.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.7e287fc1177f6b14339a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.cb6aa9a249ad29dcd58a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.2528d70ea54aa0f87758.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.4ea618025394f60cffcb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8e8af8247da73c7d3d69.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>}&lt;/script&gt;&lt;script defer="defer" src="/code/js/react-router.af76eaa9e545f56443c3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.840222d93e1c68b22ee6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/74234.fd2664df293d5ee3fc72.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3177.1f45837ebf350fcb1b06.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/18465.efca3aa84d5b1d7a0ad7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.0cc37f9d16788f81b99f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.b04da66fc7640a4a5b88.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/35017.aeeaa96fcd059dc802f3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59586.3e22eab7d3ff25b86b7f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b958de8eb80c530d128.js"&gt;&lt;/script&gt;&lt;link href="/style/css/3177.c3f17f0c40e492325ca7.css" rel="stylesheet"&gt;&lt;link href="/style/css/35017.0fa000b0b835f92c2294.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.7e97b3c950c96ab7e1af.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>